<commit_message>
feat: enhance patient data management and formatting
- Updated styles in assets/styles.css to improve UI for admin error details and ficha modal sections.
- Modified dados_pacientes.csv to include missing CPF numbers for certain patients.
- Updated dados_pacientes.xlsx to reflect changes in patient data.
- Added format.js to handle formatting of phone numbers, CPF, CNPJ, and dates in Brazilian format.
- Created a temporary file for dados_pacientes.xlsx to manage changes.
</commit_message>
<xml_diff>
--- a/dados_pacientes.xlsx
+++ b/dados_pacientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcelino/Documents/VSCODE/singular/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3C2E79F-0BEA-584D-AB7D-17C2E3A8CAAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A03A63D-23D0-3546-BFA1-B1AD3734FB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{05D45D77-41EF-8746-B47A-55222B0788A4}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="22580" xr2:uid="{05D45D77-41EF-8746-B47A-55222B0788A4}"/>
   </bookViews>
   <sheets>
     <sheet name="dados_pacientes" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="466">
   <si>
     <t xml:space="preserve">Telefone </t>
   </si>
@@ -1431,6 +1431,9 @@
   </si>
   <si>
     <t>RedesSociais</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
 </sst>
 </file>
@@ -1438,8 +1441,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="169" formatCode="[&lt;=99999999999]000\.000\.000\-00;00\.000\.000\/0000\-00"/>
-    <numFmt numFmtId="171" formatCode="\ \(##\)00000\-0000"/>
+    <numFmt numFmtId="164" formatCode="[&lt;=99999999999]000\.000\.000\-00;00\.000\.000\/0000\-00"/>
+    <numFmt numFmtId="165" formatCode="\ \(##\)00000\-0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -1483,7 +1486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1491,10 +1494,10 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1505,6 +1508,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1846,7 +1852,7 @@
     <col min="1" max="1" width="35.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.5" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="32" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -2114,7 +2120,9 @@
       <c r="C5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="3"/>
+      <c r="D5" s="3">
+        <v>11111111111</v>
+      </c>
       <c r="E5" s="4">
         <v>31973107800</v>
       </c>
@@ -2522,7 +2530,9 @@
       <c r="C13" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="D13" s="3"/>
+      <c r="D13" s="3">
+        <v>22222222222</v>
+      </c>
       <c r="E13" s="4">
         <v>31986867922</v>
       </c>
@@ -3291,6 +3301,9 @@
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>465</v>
+      </c>
       <c r="B29" s="2"/>
       <c r="C29" s="1" t="s">
         <v>273</v>
@@ -3437,7 +3450,9 @@
       <c r="C32" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D32" s="3"/>
+      <c r="D32" s="3">
+        <v>33333333333</v>
+      </c>
       <c r="E32" s="4" t="s">
         <v>309</v>
       </c>
@@ -3741,6 +3756,9 @@
       </c>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>465</v>
+      </c>
       <c r="B39" s="2"/>
       <c r="C39" s="1" t="s">
         <v>163</v>
@@ -3783,7 +3801,9 @@
       <c r="C40" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="D40" s="3"/>
+      <c r="D40" s="3">
+        <v>44444444444</v>
+      </c>
       <c r="E40" s="4" t="s">
         <v>309</v>
       </c>
@@ -3964,7 +3984,9 @@
       <c r="C44" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="D44" s="3"/>
+      <c r="D44" s="3">
+        <v>55555555555</v>
+      </c>
       <c r="E44" s="4" t="s">
         <v>309</v>
       </c>
@@ -3990,7 +4012,7 @@
       <c r="C45" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="D45" s="8" t="s">
         <v>304</v>
       </c>
       <c r="E45" s="4">

</xml_diff>